<commit_message>
May 8 24 changes IG SIC
</commit_message>
<xml_diff>
--- a/TestData/LV_T1592_ValidationsToBeCompleted.xlsx
+++ b/TestData/LV_T1592_ValidationsToBeCompleted.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E58FED8-1C8F-495C-8B8E-D3C190206FBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3D194D0-63CA-4DA9-AD04-A902A3D86A77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AddOpportunity" sheetId="1" r:id="rId1"/>
@@ -362,10 +362,10 @@
     <t>Opportunities</t>
   </si>
   <si>
-    <t>Items to complete:Info--&gt;Details--&gt;General: Client Ownership is required.Info--&gt;Details--&gt;General: Subject's Ownership is required.Info--&gt;Details--&gt;General: SIC Code is required.Info--&gt;Details--&gt;Opportunity Description: Opportunity Description is required.Fees &amp; Financials--&gt;Funds &amp; Financials: Est. Transaction Size / Market Cap (MM) is required.Fees &amp; Financials--&gt;Estimated Fees: Retainer is required. (Input zero if there's no Retainer fee.)Fees &amp; Financials--&gt;Estimated Fees: Tail Expires is required.Fees &amp; Financials--&gt;Estimated Fees: Progress/Monthly Fee is required.Fees &amp; Financials--&gt;Estimated Fees: Contingent Fee is required.Client/Subject &amp; Referral--&gt;Referral Info: Referral Contact is required.Internal Team: Team must include the following roles: Initiator, Seller, Principal, Manager, Associate(Optional), Analyst(Optional).Compliance &amp; Legal--&gt;Legal Matters: Confidentiality Agreement is required.Compliance &amp; Legal--&gt;Conflicts Check: A Conflicts Check was completed more than 30 days ago. A new Conflicts Check must be completed.Info--&gt;Administration: Estimated Close Date is required.Info--&gt;Administration: \"Women Led\" is required. Please update this field with the correct valueInfo--&gt;Administration: Fairness Opinion Component is required.Info--&gt;Administration: Date Engaged - Date of Executed Retainer or similar document.Approved NBC form - Please complete and submit this form via the NBC button.Opportunity Contacts - Add at least one Primary Opportunity Contact.Opportunity Contacts - Add at least one Billing Contact.</t>
-  </si>
-  <si>
     <t>Business Services</t>
+  </si>
+  <si>
+    <t>Items to complete:Info--&gt;Details--&gt;General: Client Ownership is required.Info--&gt;Details--&gt;General: Subject's Ownership is required.Info--&gt;Details--&gt;Opportunity Description: Opportunity Description is required.Fees &amp; Financials--&gt;Funds &amp; Financials: Est. Transaction Size / Market Cap (MM) is required.Fees &amp; Financials--&gt;Estimated Fees: Retainer is required. (Input zero if there's no Retainer fee.)Fees &amp; Financials--&gt;Estimated Fees: Tail Expires is required.Fees &amp; Financials--&gt;Estimated Fees: Progress/Monthly Fee is required.Fees &amp; Financials--&gt;Estimated Fees: Contingent Fee is required.Client/Subject &amp; Referral--&gt;Referral Info: Referral Contact is required.Internal Team: Team must include the following roles: Initiator, Seller, Principal, Manager, Associate(Optional), Analyst(Optional).Compliance &amp; Legal--&gt;Legal Matters: Confidentiality Agreement is required.Compliance &amp; Legal--&gt;Conflicts Check: A Conflicts Check was completed more than 30 days ago. A new Conflicts Check must be completed.Info--&gt;Administration: Estimated Close Date is required.Info--&gt;Administration: "Women Led" is required. Please update this field with the correct valueInfo--&gt;Administration: Fairness Opinion Component is required.Info--&gt;Administration: Date Engaged - Date of Executed Retainer or similar document.Approved NBC form - Please complete and submit this form via the NBC button.Opportunity Contacts - Add at least one Primary Opportunity Contact.Opportunity Contacts - Add at least one Billing Contact.</t>
   </si>
 </sst>
 </file>
@@ -842,7 +842,7 @@
         <v>90</v>
       </c>
       <c r="D2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E2" t="s">
         <v>7</v>
@@ -1215,9 +1215,9 @@
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:32" ht="240" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
-        <v>110</v>
+    <row r="2" spans="1:32" ht="224.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>111</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>8</v>
@@ -1314,7 +1314,8 @@
       </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.25">
-      <c r="A3" s="5"/>
+      <c r="A3" s="7"/>
+      <c r="D3" s="6"/>
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.25">
       <c r="A4" s="5"/>

</xml_diff>

<commit_message>
locators changes May 14 24 -1
</commit_message>
<xml_diff>
--- a/TestData/LV_T1592_ValidationsToBeCompleted.xlsx
+++ b/TestData/LV_T1592_ValidationsToBeCompleted.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3D194D0-63CA-4DA9-AD04-A902A3D86A77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{753E7D0A-BA9A-4DFD-83E0-F2A66FFB49AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AddOpportunity" sheetId="1" r:id="rId1"/>
@@ -53,9 +53,6 @@
     <t>AdditonalSubject</t>
   </si>
   <si>
-    <t>Dealership &amp; Rental Services</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
@@ -366,6 +363,9 @@
   </si>
   <si>
     <t>Items to complete:Info--&gt;Details--&gt;General: Client Ownership is required.Info--&gt;Details--&gt;General: Subject's Ownership is required.Info--&gt;Details--&gt;Opportunity Description: Opportunity Description is required.Fees &amp; Financials--&gt;Funds &amp; Financials: Est. Transaction Size / Market Cap (MM) is required.Fees &amp; Financials--&gt;Estimated Fees: Retainer is required. (Input zero if there's no Retainer fee.)Fees &amp; Financials--&gt;Estimated Fees: Tail Expires is required.Fees &amp; Financials--&gt;Estimated Fees: Progress/Monthly Fee is required.Fees &amp; Financials--&gt;Estimated Fees: Contingent Fee is required.Client/Subject &amp; Referral--&gt;Referral Info: Referral Contact is required.Internal Team: Team must include the following roles: Initiator, Seller, Principal, Manager, Associate(Optional), Analyst(Optional).Compliance &amp; Legal--&gt;Legal Matters: Confidentiality Agreement is required.Compliance &amp; Legal--&gt;Conflicts Check: A Conflicts Check was completed more than 30 days ago. A new Conflicts Check must be completed.Info--&gt;Administration: Estimated Close Date is required.Info--&gt;Administration: "Women Led" is required. Please update this field with the correct valueInfo--&gt;Administration: Fairness Opinion Component is required.Info--&gt;Administration: Date Engaged - Date of Executed Retainer or similar document.Approved NBC form - Please complete and submit this form via the NBC button.Opportunity Contacts - Add at least one Primary Opportunity Contact.Opportunity Contacts - Add at least one Billing Contact.</t>
+  </si>
+  <si>
+    <t>CSDN-0000001546</t>
   </si>
 </sst>
 </file>
@@ -768,153 +768,153 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="J1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="L1" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="P1" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Q1" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="S1" s="1" t="s">
-        <v>26</v>
-      </c>
       <c r="T1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="V1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="W1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="W1" s="1" t="s">
-        <v>32</v>
-      </c>
       <c r="X1" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="Y1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="Z1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="Z1" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="AA1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AB1" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E2" t="s">
+        <v>111</v>
+      </c>
+      <c r="F2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K2" t="s">
+        <v>13</v>
+      </c>
+      <c r="L2" t="s">
+        <v>15</v>
+      </c>
+      <c r="M2" t="s">
+        <v>17</v>
+      </c>
+      <c r="N2" t="s">
         <v>95</v>
       </c>
-      <c r="B2" t="s">
-        <v>95</v>
-      </c>
-      <c r="C2" t="s">
-        <v>90</v>
-      </c>
-      <c r="D2" t="s">
-        <v>110</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" t="s">
-        <v>8</v>
-      </c>
-      <c r="H2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" t="s">
-        <v>8</v>
-      </c>
-      <c r="J2" t="s">
-        <v>8</v>
-      </c>
-      <c r="K2" t="s">
-        <v>14</v>
-      </c>
-      <c r="L2" t="s">
-        <v>16</v>
-      </c>
-      <c r="M2" t="s">
-        <v>18</v>
-      </c>
-      <c r="N2" t="s">
+      <c r="O2" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="P2" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="R2" t="s">
+        <v>26</v>
+      </c>
+      <c r="S2" t="s">
+        <v>26</v>
+      </c>
+      <c r="T2" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="U2" t="s">
+        <v>29</v>
+      </c>
+      <c r="V2" t="s">
         <v>96</v>
       </c>
-      <c r="O2" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="Q2" s="3" t="s">
+      <c r="W2" t="s">
+        <v>32</v>
+      </c>
+      <c r="X2" t="s">
+        <v>34</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA2" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="R2" t="s">
-        <v>27</v>
-      </c>
-      <c r="S2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T2" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="U2" t="s">
-        <v>30</v>
-      </c>
-      <c r="V2" t="s">
-        <v>97</v>
-      </c>
-      <c r="W2" t="s">
-        <v>33</v>
-      </c>
-      <c r="X2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>48</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>43</v>
-      </c>
-      <c r="AA2" s="3" t="s">
-        <v>101</v>
-      </c>
       <c r="AB2" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -934,15 +934,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -960,12 +960,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
   </sheetData>
@@ -980,12 +980,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -1011,75 +1011,75 @@
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="9" t="s">
-        <v>37</v>
-      </c>
       <c r="C1" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G1" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="E1" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>52</v>
-      </c>
       <c r="H1" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I1" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="J1" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>93</v>
-      </c>
-      <c r="K1" s="9" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="162" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E2" s="8" t="s">
         <v>0</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>0</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="K2" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L2" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -1119,198 +1119,198 @@
   <sheetData>
     <row r="1" spans="1:32" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="C1" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="C1" s="9" t="s">
-        <v>58</v>
-      </c>
       <c r="D1" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="E1" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="F1" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="L1" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="M1" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="N1" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="N1" s="10" t="s">
+      <c r="O1" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="P1" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="Q1" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="R1" s="9" t="s">
         <v>72</v>
-      </c>
-      <c r="Q1" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="R1" s="9" t="s">
-        <v>73</v>
       </c>
       <c r="S1" s="9" t="s">
         <v>0</v>
       </c>
       <c r="T1" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="U1" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="V1" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="W1" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="W1" s="9" t="s">
+      <c r="X1" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="X1" s="9" t="s">
+      <c r="Y1" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="Y1" s="9" t="s">
+      <c r="Z1" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="Z1" s="9" t="s">
-        <v>82</v>
-      </c>
       <c r="AA1" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="AB1" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="AB1" s="9" t="s">
+      <c r="AC1" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="AC1" s="9" t="s">
+      <c r="AD1" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="AD1" s="9" t="s">
+      <c r="AE1" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="AE1" s="9" t="s">
+      <c r="AF1" s="9" t="s">
         <v>88</v>
-      </c>
-      <c r="AF1" s="9" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:32" ht="224.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J2" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="L2" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M2" s="8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="O2" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="P2" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Q2" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R2" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="S2" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="T2" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="U2" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V2" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="W2" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="X2" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="Y2" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="Z2" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AA2" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AB2" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AC2" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AD2" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AE2" s="8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AF2" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
July 5 changes 1
</commit_message>
<xml_diff>
--- a/TestData/LV_T1592_ValidationsToBeCompleted.xlsx
+++ b/TestData/LV_T1592_ValidationsToBeCompleted.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA1761A-A0BF-444A-9746-E994C589E80D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B93F413-B57F-497D-B0DE-02A464B8D5EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -365,7 +365,7 @@
     <t>CSDN-0000001546</t>
   </si>
   <si>
-    <t>Items to complete:Info--&gt;Details--&gt;General: Client Ownership is required.Info--&gt;Details--&gt;General: Subject's Ownership is required.Info--&gt;Details--&gt;Opportunity Description: Opportunity Description is required.Fees &amp; Financials--&gt;Funds &amp; Financials: Est. Transaction Size / Market Cap (MM) is required.Fees &amp; Financials--&gt;Estimated Fees: Retainer is required. (Input zero if there's no Retainer fee.)Fees &amp; Financials--&gt;Estimated Fees: Tail Expires is required.Fees &amp; Finances--&gt;Estimated Fees: Shared Services Expense is required.Fees &amp; Financials--&gt;Estimated Fees: Expense Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Legal Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Progress/Monthly Fee is required.Fees &amp; Financials--&gt;Estimated Fees: Contingent Fee is required.Compliance &amp; Legal--&gt;Legal Matters: Indemnification Language is required.Client/Subject &amp; Referral--&gt;Referral Info: Referral Contact is required.Internal Team: Team must include the following roles: Initiator, Seller, Principal, Manager, Associate(Optional), Analyst(Optional).Compliance &amp; Legal--&gt;Legal Matters: Confidentiality Agreement is required.Compliance &amp; Legal--&gt;Conflicts Check: A Conflicts Check was completed more than 30 days ago. A new Conflicts Check must be completed.Info--&gt;Administration: Estimated Close Date is required.Info--&gt;Administration: "Women Led" is required. Please update this field with the correct valueInfo--&gt;Administration: Fairness Opinion Component is required.Info--&gt;Administration: Date Engaged - Date of Executed Retainer or similar document.Approved NBC form - Please complete and submit this form via the NBC button.Opportunity Contacts - Add at least one Primary Opportunity Contact.Opportunity Contacts - Add at least one Billing Contact.</t>
+    <t>Items to complete:Info--&gt;Details--&gt;General: Client Ownership is required.Info--&gt;Details--&gt;General: Subject's Ownership is required.Info--&gt;Details--&gt;Opportunity Description: Opportunity Description is required.Fees &amp; Financials--&gt;Funds &amp; Financials: Est. Transaction Size / Market Cap (MM) is required.Fees &amp; Financials--&gt;Estimated Fees: Retainer is required. (Input zero if there's no Retainer fee.)Fees &amp; Financials--&gt;Estimated Fees: Tail Expires is required.Fees &amp; Financials--&gt;Estimated Fees: Shared Services Expense is required.Fees &amp; Financials--&gt;Estimated Fees: Expense Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Legal Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Progress/Monthly Fee is required.Fees &amp; Financials--&gt;Estimated Fees: Contingent Fee is required.Compliance &amp; Legal--&gt;Legal Matters: Indemnification Language is required.Client/Subject &amp; Referral--&gt;Referral Info: Referral Contact is required.Internal Team: Team must include the following roles: Initiator, Seller, Principal, Manager, Associate(Optional), Analyst(Optional).Compliance &amp; Legal--&gt;Legal Matters: Confidentiality Agreement is required.Compliance &amp; Legal--&gt;Conflicts Check: A Conflicts Check was completed more than 30 days ago. A new Conflicts Check must be completed.Info--&gt;Administration: Estimated Close Date is required.Info--&gt;Administration: "Women Led" is required. Please update this field with the correct valueInfo--&gt;Administration: Fairness Opinion Component is required.Info--&gt;Administration: Date Engaged - Date of Executed Retainer or similar document.Approved NBC form - Please complete and submit this form via the NBC button.Opportunity Contacts - Add at least one Primary Opportunity Contact.Opportunity Contacts - Add at least one Billing Contact.</t>
   </si>
 </sst>
 </file>
@@ -1313,7 +1313,8 @@
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:32" ht="254.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="7"/>
       <c r="D3" s="6"/>
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
May 5 2025 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_T1592_ValidationsToBeCompleted.xlsx
+++ b/TestData/LV_T1592_ValidationsToBeCompleted.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{834BF522-4D3F-40EF-BCE6-3153CC939D90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F36624B4-5492-4775-A439-22C74510FD86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
@@ -365,7 +365,7 @@
     <t>BUS - Business Services</t>
   </si>
   <si>
-    <t>Items to complete:Info--&gt;Details--&gt;General: Client Ownership is required.Info--&gt;Details--&gt;General: Subject's Ownership is required.Info--&gt;Details--&gt;Opportunity Description: Opportunity Description is required.Fees &amp; Financials--&gt;Funds &amp; Financials: Est. Transaction Size / Market Cap (MM) is required.Fees &amp; Financials--&gt;Estimated Fees: Retainer is required. (Input zero if there's no Retainer fee.)Fees &amp; Financials--&gt;Estimated Fees: Shared Services Expense is required.Fees &amp; Financials--&gt;Estimated Fees: Expense Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Legal Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Progress/Monthly Fee is required.Fees &amp; Financials--&gt;Estimated Fees: Contingent Fee is required.Compliance &amp; Legal--&gt;Legal Matters: Indemnification Language is required.Client/Subject &amp; Referral--&gt;Referral Info: Referral Contact is required.Internal Team: Team must include the following roles: Initiator, Seller, Principal, Manager, Associate(Optional), Analyst(Optional).Compliance &amp; Legal--&gt;Legal Matters: Confidentiality Agreement is required.Compliance &amp; Legal--&gt;Conflicts Check: A Conflicts Check was completed more than 30 days ago. A new Conflicts Check must be completed.Info--&gt;Administration: Estimated Close Date is required.Info--&gt;Administration: "Women Led" is required. Please update this field with the correct valueInfo--&gt;Administration: Fairness Opinion Component is required.Info--&gt;Administration: Date Engaged - Date of Executed Retainer or similar document.Approved NBC form - Please complete and submit this form via the NBC button.Opportunity Contacts - Add at least one Primary Opportunity Contact.Opportunity Contacts - Add at least one Billing Contact.</t>
+    <t>Items to complete:Info--&gt;Details--&gt;General: Client Ownership is required.Info--&gt;Details--&gt;General: Subject's Ownership is required.Info--&gt;Details--&gt;Opportunity Description: Opportunity Description is required.Fees &amp; Financials--&gt;Funds &amp; Financials: Est. Transaction Size / Market Cap (MM) is required.Fees &amp; Financials--&gt;Estimated Fees: Retainer is required. (Input zero if there's no Retainer fee.)Fees &amp; Financials--&gt;Estimated Fees: Shared Services Expense is required.Fees &amp; Financials--&gt;Estimated Fees: Expense Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Legal Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Progress/Monthly Fee is required.Fees &amp; Financials--&gt;Estimated Fees: Contingent Fee is required.Compliance &amp; Legal--&gt;Legal Matters: Indemnification Language is required.Client/Subject &amp; Referral--&gt;Referral Info: Referral Contact is required.Internal Team: Team must include the following roles: Initiator, Seller, Principal, Manager, Associate(Optional), Analyst(Optional).Compliance &amp; Legal--&gt;Legal Matters: Confidentiality Agreement is required.Compliance &amp; Legal--&gt;Conflicts Check: A Conflicts Check was completed more than 30 days ago. A new Conflicts Check must be completed.Info--&gt;Administration: Location where Service Benefit was provided is required.Info--&gt;Administration: Estimated Close Date is required.Info--&gt;Administration: "Women Led" is required. Please update this field with the correct valueInfo--&gt;Administration: Fairness Opinion Component is required.Info--&gt;Administration: Date Engaged - Date of Executed Retainer or similar document.Approved NBC form - Please complete and submit this form via the NBC button.Opportunity Contacts - Add at least one Primary Opportunity Contact.Opportunity Contacts - Add at least one Billing Contact.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
req field's validation may 152025
</commit_message>
<xml_diff>
--- a/TestData/LV_T1592_ValidationsToBeCompleted.xlsx
+++ b/TestData/LV_T1592_ValidationsToBeCompleted.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F36624B4-5492-4775-A439-22C74510FD86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F1FCC48-8EEC-4FF0-8B2E-16DA13AA3CB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -365,7 +365,7 @@
     <t>BUS - Business Services</t>
   </si>
   <si>
-    <t>Items to complete:Info--&gt;Details--&gt;General: Client Ownership is required.Info--&gt;Details--&gt;General: Subject's Ownership is required.Info--&gt;Details--&gt;Opportunity Description: Opportunity Description is required.Fees &amp; Financials--&gt;Funds &amp; Financials: Est. Transaction Size / Market Cap (MM) is required.Fees &amp; Financials--&gt;Estimated Fees: Retainer is required. (Input zero if there's no Retainer fee.)Fees &amp; Financials--&gt;Estimated Fees: Shared Services Expense is required.Fees &amp; Financials--&gt;Estimated Fees: Expense Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Legal Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Progress/Monthly Fee is required.Fees &amp; Financials--&gt;Estimated Fees: Contingent Fee is required.Compliance &amp; Legal--&gt;Legal Matters: Indemnification Language is required.Client/Subject &amp; Referral--&gt;Referral Info: Referral Contact is required.Internal Team: Team must include the following roles: Initiator, Seller, Principal, Manager, Associate(Optional), Analyst(Optional).Compliance &amp; Legal--&gt;Legal Matters: Confidentiality Agreement is required.Compliance &amp; Legal--&gt;Conflicts Check: A Conflicts Check was completed more than 30 days ago. A new Conflicts Check must be completed.Info--&gt;Administration: Location where Service Benefit was provided is required.Info--&gt;Administration: Estimated Close Date is required.Info--&gt;Administration: "Women Led" is required. Please update this field with the correct valueInfo--&gt;Administration: Fairness Opinion Component is required.Info--&gt;Administration: Date Engaged - Date of Executed Retainer or similar document.Approved NBC form - Please complete and submit this form via the NBC button.Opportunity Contacts - Add at least one Primary Opportunity Contact.Opportunity Contacts - Add at least one Billing Contact.</t>
+    <t>Items to complete:Info--&gt;Details--&gt;General: Client Ownership is required.Info--&gt;Details--&gt;General: Subject's Ownership is required.Info--&gt;Details--&gt;Opportunity Description: Opportunity Description is required.Fees &amp; Financials--&gt;Funds &amp; Financials: Est. Transaction Size / Market Cap (MM) is required.Fees &amp; Financials--&gt;Estimated Fees: Retainer is required. (Input zero if there's no Retainer fee.)Fees &amp; Financials--&gt;Estimated Fees: Shared Services Expense is required.Fees &amp; Financials--&gt;Estimated Fees: Expense Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Legal Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Progress/Monthly Fee is required.Fees &amp; Financials--&gt;Estimated Fees: Contingent Fee is required.Compliance &amp; Legal--&gt;Legal Matters: Indemnification Language is required.Client/Subject &amp; Referral--&gt;Referral Info: Referral Contact is required.Internal Team: Team must include the following roles: Initiator, Seller, Principal, Manager, Associate(Optional), Analyst(Optional).Compliance &amp; Legal--&gt;Legal Matters: Confidentiality Agreement is required.Compliance &amp; Legal--&gt;Conflicts Check: A Conflicts Check was completed more than 30 days ago. A new Conflicts Check must be completed.Info--&gt;Administration: Location where Benefit is to be Provided is required.Info--&gt;Administration: Estimated Close Date is required.Info--&gt;Administration: "Women Led" is required. Please update this field with the correct valueInfo--&gt;Administration: Fairness Opinion Component is required.Info--&gt;Administration: Date Engaged - Date of Executed Retainer or similar document.Approved NBC form - Please complete and submit this form via the NBC button.Opportunity Contacts - Add at least one Primary Opportunity Contact.Opportunity Contacts - Add at least one Billing Contact.</t>
   </si>
 </sst>
 </file>
@@ -722,13 +722,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>19</v>
       </c>
@@ -736,7 +736,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>104</v>
       </c>
@@ -749,17 +749,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8244481F-F1B5-4BC7-BE8A-260AA0DF5D37}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>106</v>
       </c>
@@ -772,14 +772,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FB45B32-4FF3-421E-8C03-B189CD186655}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>108</v>
       </c>
@@ -792,31 +792,31 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AB2"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.5546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="14.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="14.5546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="14.5546875" style="4" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="21" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="27" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.28515625" customWidth="1"/>
+    <col min="26" max="26" width="11.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -902,7 +902,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>94</v>
       </c>
@@ -997,20 +997,20 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="86.7109375" customWidth="1"/>
+    <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="86.6640625" customWidth="1"/>
     <col min="10" max="10" width="45" customWidth="1"/>
-    <col min="11" max="11" width="54.42578125" customWidth="1"/>
+    <col min="11" max="11" width="54.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>35</v>
       </c>
@@ -1045,7 +1045,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="162" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="162" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
         <v>96</v>
       </c>
@@ -1092,33 +1092,33 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:AF33"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="95.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.140625" style="8" customWidth="1"/>
-    <col min="7" max="7" width="8.85546875" style="8"/>
-    <col min="8" max="8" width="12.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="12" width="8.85546875" style="8"/>
-    <col min="13" max="13" width="10.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.85546875" style="3"/>
-    <col min="15" max="16" width="8.85546875" style="8"/>
-    <col min="17" max="17" width="10.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="29.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="8.85546875" style="8"/>
-    <col min="21" max="21" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="8.85546875" style="8"/>
-    <col min="23" max="23" width="13.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="24" max="30" width="8.85546875" style="8"/>
-    <col min="31" max="31" width="10.5703125" style="8" customWidth="1"/>
-    <col min="32" max="32" width="102.28515625" style="8" customWidth="1"/>
-    <col min="33" max="16384" width="8.85546875" style="8"/>
+    <col min="1" max="1" width="95.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.109375" style="8" customWidth="1"/>
+    <col min="7" max="7" width="8.88671875" style="8"/>
+    <col min="8" max="8" width="12.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="12" width="8.88671875" style="8"/>
+    <col min="13" max="13" width="10.33203125" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.88671875" style="3"/>
+    <col min="15" max="16" width="8.88671875" style="8"/>
+    <col min="17" max="17" width="10.44140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="29.5546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="8.88671875" style="8"/>
+    <col min="21" max="21" width="9.88671875" style="8" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="8.88671875" style="8"/>
+    <col min="23" max="23" width="13.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="24" max="30" width="8.88671875" style="8"/>
+    <col min="31" max="31" width="10.5546875" style="8" customWidth="1"/>
+    <col min="32" max="32" width="102.33203125" style="8" customWidth="1"/>
+    <col min="33" max="16384" width="8.88671875" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" s="9" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:32" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>55</v>
       </c>
@@ -1216,7 +1216,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="2" spans="1:32" ht="247.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:32" ht="247.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="7" t="s">
         <v>111</v>
       </c>
@@ -1314,98 +1314,98 @@
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:32" ht="254.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:32" ht="254.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7"/>
       <c r="D3" s="6"/>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A4" s="5"/>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
     </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A6" s="5"/>
     </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A7" s="5"/>
     </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A8" s="5"/>
     </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
     </row>
-    <row r="10" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A10" s="5"/>
     </row>
-    <row r="11" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
     </row>
-    <row r="12" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
     </row>
-    <row r="13" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
     </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
     </row>
-    <row r="15" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A15" s="5"/>
     </row>
-    <row r="16" spans="1:32" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:32" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
     </row>
-    <row r="17" spans="1:1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="5"/>
     </row>
-    <row r="18" spans="1:1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5"/>
     </row>
-    <row r="19" spans="1:1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="5"/>
     </row>
-    <row r="20" spans="1:1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5"/>
     </row>
-    <row r="21" spans="1:1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="5"/>
     </row>
-    <row r="22" spans="1:1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5"/>
     </row>
-    <row r="23" spans="1:1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="5"/>
     </row>
-    <row r="24" spans="1:1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="5"/>
     </row>
-    <row r="25" spans="1:1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5"/>
     </row>
-    <row r="26" spans="1:1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5"/>
     </row>
-    <row r="27" spans="1:1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="5"/>
     </row>
-    <row r="28" spans="1:1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="5"/>
     </row>
-    <row r="29" spans="1:1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5"/>
     </row>
-    <row r="30" spans="1:1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5"/>
     </row>
-    <row r="31" spans="1:1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5"/>
     </row>
-    <row r="32" spans="1:1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5"/>
     </row>
-    <row r="33" spans="1:1" ht="14.45" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="5"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sept 16 2025 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_T1592_ValidationsToBeCompleted.xlsx
+++ b/TestData/LV_T1592_ValidationsToBeCompleted.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{875A3993-86DE-4701-A7B8-9C1D7B432BF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{934D9F44-F155-4195-A87B-97494B3BE91E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="2" r:id="rId1"/>
@@ -362,10 +362,10 @@
     <t>BUS - Business Services</t>
   </si>
   <si>
-    <t>Items to complete:Info--&gt;Details--&gt;General: Client Ownership is required.Info--&gt;Details--&gt;General: Subject's Ownership is required.Info--&gt;Details--&gt;Opportunity Description: Opportunity Description is required.Fees &amp; Financials--&gt;Funds &amp; Financials: Est. Transaction Size / Market Cap (MM) is required.Fees &amp; Financials--&gt;Estimated Fees: Retainer is required. (Input zero if there's no Retainer fee.)Fees &amp; Financials--&gt;Estimated Fees: Shared Services Expense is required.Fees &amp; Financials--&gt;Estimated Fees: Expense Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Legal Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Progress/Monthly Fee is required.Fees &amp; Financials--&gt;Estimated Fees: Contingent Fee is required.Compliance &amp; Legal--&gt;Legal Matters: Indemnification Language is required.Client/Subject &amp; Referral--&gt;Referral Info: Referral Contact is required.Internal Team: Team must include the following roles: Initiator, Seller, Principal, Manager, Associate(Optional), Analyst(Optional).Compliance &amp; Legal--&gt;Legal Matters: Confidentiality Agreement is required.Compliance &amp; Legal--&gt;Conflicts Check: A Conflicts Check was completed more than 30 days ago. A new Conflicts Check must be completed.Info--&gt;Administration: Location where Benefit is to be Provided is required.Info--&gt;Administration: Estimated Close Date is required.Info--&gt;Administration: "Women Led" is required. Please update this field with the correct valueInfo--&gt;Administration: Fairness Opinion Component is required.Info--&gt;Administration: Date Engaged - Date of Executed Retainer or similar document.Approved NBC form - Please complete and submit this form via the NBC button.Opportunity Contacts - Add at least one Primary Opportunity Contact.Opportunity Contacts - Add at least one Billing Contact.</t>
-  </si>
-  <si>
     <t>Debt Financing</t>
+  </si>
+  <si>
+    <t>Items to complete:Info--&gt;Details--&gt;General: Client Ownership is required.Info--&gt;Details--&gt;General: Subject's Ownership is required.Info--&gt;Details--&gt;Opportunity Description: Opportunity Description is required.Fees &amp; Financials--&gt;Funds &amp; Financials: Est. Transaction Size / Market Cap (MM) is required.Fees &amp; Financials--&gt;Estimated Fees: Retainer is required. (Input zero if there's no Retainer fee.)Fees &amp; Financials--&gt;Estimated Fees: Shared Services Expense is required.Fees &amp; Financials--&gt;Estimated Fees: Expense Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Legal Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Progress/Monthly Fee is required.Fees &amp; Financials--&gt;Estimated Fees: Contingent Fee is required.Compliance &amp; Legal--&gt;Legal Matters: Indemnification Language is required.KYC/Client/Subject/Referra--&gt;Referral Info: Referral Contact is required.Internal Team: Team must include the following roles: Initiator, Seller, Principal, Manager, Associate(Optional), Analyst(Optional).Compliance &amp; Legal--&gt;Legal Matters: Confidentiality Agreement is required.Compliance &amp; Legal--&gt;Conflicts Check: A Conflicts Check was completed more than 30 days ago. A new Conflicts Check must be completed.Info--&gt;Administration: Location where Benefit is to be Provided is required.Info--&gt;Administration: Estimated Close Date is required.Info--&gt;Administration: "Women Led" is required. Please update this field with the correct valueInfo--&gt;Administration: Fairness Opinion Component is required.Info--&gt;Administration: Date Engaged - Date of Executed Retainer or similar document.Approved NBC form - Please complete and submit this form via the NBC button.Opportunity Contacts - Add at least one Primary Opportunity Contact.Opportunity Contacts - Add at least one Billing Contact.</t>
   </si>
 </sst>
 </file>
@@ -910,7 +910,7 @@
         <v>93</v>
       </c>
       <c r="C2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D2" t="s">
         <v>109</v>
@@ -1218,7 +1218,7 @@
     </row>
     <row r="2" spans="1:32" ht="247.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
KYC changes Sept 16 2025
</commit_message>
<xml_diff>
--- a/TestData/LV_T1592_ValidationsToBeCompleted.xlsx
+++ b/TestData/LV_T1592_ValidationsToBeCompleted.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{934D9F44-F155-4195-A87B-97494B3BE91E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C117572-909B-4787-948F-62A07C72CFB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -365,7 +365,7 @@
     <t>Debt Financing</t>
   </si>
   <si>
-    <t>Items to complete:Info--&gt;Details--&gt;General: Client Ownership is required.Info--&gt;Details--&gt;General: Subject's Ownership is required.Info--&gt;Details--&gt;Opportunity Description: Opportunity Description is required.Fees &amp; Financials--&gt;Funds &amp; Financials: Est. Transaction Size / Market Cap (MM) is required.Fees &amp; Financials--&gt;Estimated Fees: Retainer is required. (Input zero if there's no Retainer fee.)Fees &amp; Financials--&gt;Estimated Fees: Shared Services Expense is required.Fees &amp; Financials--&gt;Estimated Fees: Expense Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Legal Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Progress/Monthly Fee is required.Fees &amp; Financials--&gt;Estimated Fees: Contingent Fee is required.Compliance &amp; Legal--&gt;Legal Matters: Indemnification Language is required.KYC/Client/Subject/Referra--&gt;Referral Info: Referral Contact is required.Internal Team: Team must include the following roles: Initiator, Seller, Principal, Manager, Associate(Optional), Analyst(Optional).Compliance &amp; Legal--&gt;Legal Matters: Confidentiality Agreement is required.Compliance &amp; Legal--&gt;Conflicts Check: A Conflicts Check was completed more than 30 days ago. A new Conflicts Check must be completed.Info--&gt;Administration: Location where Benefit is to be Provided is required.Info--&gt;Administration: Estimated Close Date is required.Info--&gt;Administration: "Women Led" is required. Please update this field with the correct valueInfo--&gt;Administration: Fairness Opinion Component is required.Info--&gt;Administration: Date Engaged - Date of Executed Retainer or similar document.Approved NBC form - Please complete and submit this form via the NBC button.Opportunity Contacts - Add at least one Primary Opportunity Contact.Opportunity Contacts - Add at least one Billing Contact.</t>
+    <t>Items to complete:Info--&gt;Details--&gt;General: Client Ownership is required.Info--&gt;Details--&gt;General: Subject's Ownership is required.Info--&gt;Details--&gt;Opportunity Description: Opportunity Description is required.Fees &amp; Financials--&gt;Funds &amp; Financials: Est. Transaction Size / Market Cap (MM) is required.Fees &amp; Financials--&gt;Estimated Fees: Retainer is required. (Input zero if there's no Retainer fee.)Fees &amp; Financials--&gt;Estimated Fees: Shared Services Expense is required.Fees &amp; Financials--&gt;Estimated Fees: Expense Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Legal Cap is required.Fees &amp; Financials--&gt;Estimated Fees: Progress/Monthly Fee is required.Fees &amp; Financials--&gt;Estimated Fees: Contingent Fee is required.Compliance &amp; Legal--&gt;Legal Matters: Indemnification Language is required.KYC/Client/Subject/Referral--&gt;Referral Info: Referral Contact is required.Internal Team: Team must include the following roles: Initiator, Seller, Principal, Manager, Associate(Optional), Analyst(Optional).Compliance &amp; Legal--&gt;Legal Matters: Confidentiality Agreement is required.Compliance &amp; Legal--&gt;Conflicts Check: A Conflicts Check was completed more than 30 days ago. A new Conflicts Check must be completed.Info--&gt;Administration: Location where Benefit is to be Provided is required.Info--&gt;Administration: Estimated Close Date is required.Info--&gt;Administration: "Women Led" is required. Please update this field with the correct valueInfo--&gt;Administration: Fairness Opinion Component is required.Info--&gt;Administration: Date Engaged - Date of Executed Retainer or similar document.Approved NBC form - Please complete and submit this form via the NBC button.Opportunity Contacts - Add at least one Primary Opportunity Contact.Opportunity Contacts - Add at least one Billing Contact.</t>
   </si>
 </sst>
 </file>

</xml_diff>